<commit_message>
lab 5 data stuff
</commit_message>
<xml_diff>
--- a/Fall 2025/Aero Design 1/Trade Studies/Microcontroller Trade Study.xlsx
+++ b/Fall 2025/Aero Design 1/Trade Studies/Microcontroller Trade Study.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noahtouchton/School_Git/School/Fall 2025/Aero Design 1/Trade Studies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5237F53-45CF-9F4F-A5B1-3155190ED278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{56294D5C-0A06-004E-9FE2-73E2091C3C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="800" windowWidth="27160" windowHeight="20960" xr2:uid="{CBE0DF9F-DDFE-4833-8F35-1B1A204C32DC}"/>
+    <workbookView xWindow="4420" yWindow="900" windowWidth="27160" windowHeight="20960" xr2:uid="{CBE0DF9F-DDFE-4833-8F35-1B1A204C32DC}"/>
   </bookViews>
   <sheets>
     <sheet name="TS" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="49">
   <si>
     <t>Part:</t>
   </si>
@@ -196,55 +196,43 @@
     <t>(Group 4)</t>
   </si>
   <si>
+    <t>Noah Touchton</t>
+  </si>
+  <si>
+    <t>Communications</t>
+  </si>
+  <si>
+    <t>Power Consumption</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
     <t>Microcontroller</t>
   </si>
   <si>
-    <t>Noah Touchton</t>
-  </si>
-  <si>
-    <t>Communications</t>
-  </si>
-  <si>
-    <t>Reliability</t>
-  </si>
-  <si>
-    <t>Compute performance</t>
-  </si>
-  <si>
-    <t>Interfaces &amp; I/O</t>
-  </si>
-  <si>
-    <t>Memory &amp; storage</t>
-  </si>
-  <si>
-    <t>RTOS &amp; driver support</t>
-  </si>
-  <si>
-    <t>Power efficiency</t>
-  </si>
-  <si>
-    <t>Dev ecosystem/tooling</t>
-  </si>
-  <si>
-    <t>Cost &amp; lead time</t>
-  </si>
-  <si>
-    <t>Form factor/integration</t>
-  </si>
-  <si>
-    <t>STM32H7 (Cortex-M7 @ 400–480 MHz)</t>
-  </si>
-  <si>
-    <t>STM32L5 (Cortex-M33 low-power)</t>
-  </si>
-  <si>
-    <t>Microchip SAMRH71 (rad-tolerant M7)</t>
-  </si>
-  <si>
-    <t>Teensy 4.1 (i.MX RT1062, 600 MHz)</t>
-  </si>
-  <si>
-    <t>ESP32-S3 (dual-core Wi-Fi/BLE)</t>
+    <t>Radiation Tolerance</t>
+  </si>
+  <si>
+    <t>TID</t>
+  </si>
+  <si>
+    <t>Processing Performance</t>
+  </si>
+  <si>
+    <t>1 to 10</t>
+  </si>
+  <si>
+    <t>3D Plus Fusio RT</t>
+  </si>
+  <si>
+    <t>Gom Space A3200</t>
+  </si>
+  <si>
+    <t>AAC Clyde Sirius</t>
   </si>
 </sst>
 </file>
@@ -698,46 +686,46 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -746,7 +734,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -821,14 +809,20 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -845,19 +839,19 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -890,24 +884,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -917,13 +893,10 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1279,111 +1252,99 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC4302AA-4CFD-4C9C-A5EA-EC60A679F4CF}">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.1640625" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="3" customWidth="1"/>
+    <col min="2" max="2" width="15.5" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="5" width="14.5" customWidth="1"/>
     <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.1640625" customWidth="1"/>
-    <col min="8" max="8" width="13.5" customWidth="1"/>
-    <col min="13" max="13" width="13.83203125" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" customWidth="1"/>
-    <col min="15" max="15" width="10" customWidth="1"/>
+    <col min="7" max="8" width="10.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="45"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B1" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="47"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="46" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="47"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B2" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="49"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="46" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="47"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B3" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="49"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="48">
+      <c r="B4" s="50">
         <v>45916</v>
       </c>
-      <c r="C4" s="49"/>
-    </row>
-    <row r="5" spans="1:20" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="50" t="s">
+      <c r="C4" s="51"/>
+    </row>
+    <row r="5" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="39"/>
+      <c r="B5" s="38"/>
       <c r="C5" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
       <c r="E8" s="11"/>
     </row>
-    <row r="9" spans="1:20" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="33" t="s">
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="41"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" s="33"/>
+      <c r="K9" s="34"/>
+      <c r="L9" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="G9" s="34"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="30" t="s">
-        <v>49</v>
-      </c>
-      <c r="J9" s="31"/>
-      <c r="K9" s="32"/>
-      <c r="L9" s="33" t="s">
-        <v>50</v>
-      </c>
-      <c r="M9" s="34"/>
-      <c r="N9" s="35"/>
-      <c r="O9" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="P9" s="37"/>
-      <c r="Q9" s="38"/>
-      <c r="R9" s="33" t="s">
-        <v>52</v>
-      </c>
-      <c r="S9" s="34"/>
-      <c r="T9" s="35"/>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B10" s="51" t="s">
+      <c r="M9" s="36"/>
+      <c r="N9" s="37"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B10" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="52"/>
+      <c r="C10" s="28" t="s">
+        <v>7</v>
+      </c>
       <c r="D10" s="16" t="s">
         <v>6</v>
       </c>
@@ -1417,166 +1378,110 @@
       <c r="N10" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="O10" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="P10" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q10" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="R10" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="S10" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="T10" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B11" s="53" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="54"/>
-      <c r="D11" s="23">
-        <v>20</v>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B11" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="22">
+        <v>25</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="5">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G11" s="24">
-        <f t="shared" ref="G11:G12" si="0">IF($E11="Y", F11/SUM($F11,$I11,$L11,$O11,$R11), (1/F11)/SUM(1/$F11,1/$I11,1/$L11,1/$O11,1/$R11))</f>
-        <v>0.21052631578947367</v>
+        <f>IF($E11="Y", F11/SUM($F11,$I11,$L11), (1/F11)/SUM(1/$F11,1/$I11,1/$L11))</f>
+        <v>6.6666666666666666E-2</v>
       </c>
       <c r="H11" s="10">
-        <f>G11*$D11</f>
-        <v>4.2105263157894735</v>
+        <f>G11*D11</f>
+        <v>1.6666666666666667</v>
       </c>
       <c r="I11" s="5">
+        <v>40</v>
+      </c>
+      <c r="J11" s="24">
+        <f>IF($E11="Y", I11/SUM($F11,$I11,$L11), (1/I11)/SUM(1/$F11,1/$I11,1/$L11))</f>
+        <v>0.26666666666666666</v>
+      </c>
+      <c r="K11" s="10">
+        <f>J11*D11</f>
+        <v>6.666666666666667</v>
+      </c>
+      <c r="L11" s="5">
+        <v>100</v>
+      </c>
+      <c r="M11" s="24">
+        <f>IF($E11="Y", L11/SUM($F11,$I11,$L11), (1/L11)/SUM(1/$F11,1/$I11,1/$L11))</f>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="N11" s="10">
+        <f>M11*D11</f>
+        <v>16.666666666666664</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B12" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="24">
+        <v>30</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="5">
+        <v>1.8</v>
+      </c>
+      <c r="G12" s="24">
+        <f t="shared" ref="G12:G14" si="0">IF($E12="Y", F12/SUM($F12,$I12,$L12), (1/F12)/SUM(1/$F12,1/$I12,1/$L12))</f>
+        <v>0.4</v>
+      </c>
+      <c r="H12" s="10">
+        <f t="shared" ref="H12:H14" si="1">G12*D12</f>
+        <v>12</v>
+      </c>
+      <c r="I12" s="5">
+        <v>2</v>
+      </c>
+      <c r="J12" s="24">
+        <f t="shared" ref="J12:J14" si="2">IF($E12="Y", I12/SUM($F12,$I12,$L12), (1/I12)/SUM(1/$F12,1/$I12,1/$L12))</f>
+        <v>0.36</v>
+      </c>
+      <c r="K12" s="10">
+        <f t="shared" ref="K12:K14" si="3">J12*D12</f>
+        <v>10.799999999999999</v>
+      </c>
+      <c r="L12" s="5">
         <v>3</v>
       </c>
-      <c r="J11" s="24">
-        <f t="shared" ref="J11:J12" si="1">IF($E11="Y", I11/SUM($F11,$I11,$L11,$O11,$R11), (1/I11)/SUM(1/$F11,1/$I11,1/$L11,1/$O11,1/$R11))</f>
-        <v>0.15789473684210525</v>
-      </c>
-      <c r="K11" s="10">
-        <f>J11*$D11</f>
-        <v>3.1578947368421053</v>
-      </c>
-      <c r="L11" s="5">
-        <v>3</v>
-      </c>
-      <c r="M11" s="24">
-        <f t="shared" ref="M11:M12" si="2">IF($E11="Y", L11/SUM($F11,$I11,$L11,$O11,$R11), (1/L11)/SUM(1/$F11,1/$I11,1/$L11,1/$O11,1/$R11))</f>
-        <v>0.15789473684210525</v>
-      </c>
-      <c r="N11" s="10">
-        <f>M11*$D11</f>
-        <v>3.1578947368421053</v>
-      </c>
-      <c r="O11" s="5">
-        <v>5</v>
-      </c>
-      <c r="P11" s="24">
-        <f t="shared" ref="P11:P12" si="3">IF($E11="Y", O11/SUM($F11,$I11,$L11,$O11,$R11), (1/O11)/SUM(1/$F11,1/$I11,1/$L11,1/$O11,1/$R11))</f>
-        <v>0.26315789473684209</v>
-      </c>
-      <c r="Q11" s="10">
-        <f>P11*$D11</f>
-        <v>5.2631578947368416</v>
-      </c>
-      <c r="R11" s="5">
-        <v>4</v>
-      </c>
-      <c r="S11" s="24">
-        <f t="shared" ref="S11:S12" si="4">IF($E11="Y", R11/SUM($F11,$I11,$L11,$O11,$R11), (1/R11)/SUM(1/$F11,1/$I11,1/$L11,1/$O11,1/$R11))</f>
-        <v>0.21052631578947367</v>
-      </c>
-      <c r="T11" s="10">
-        <f>S11*$D11</f>
-        <v>4.2105263157894735</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B12" s="55" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" s="56"/>
-      <c r="D12" s="23">
-        <v>15</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="5">
-        <v>5</v>
-      </c>
-      <c r="G12" s="24">
-        <f t="shared" si="0"/>
-        <v>0.23809523809523808</v>
-      </c>
-      <c r="H12" s="10">
-        <f t="shared" ref="H12:H19" si="5">G12*$D12</f>
-        <v>3.5714285714285712</v>
-      </c>
-      <c r="I12" s="5">
-        <v>4</v>
-      </c>
-      <c r="J12" s="24">
-        <f t="shared" si="1"/>
-        <v>0.19047619047619047</v>
-      </c>
-      <c r="K12" s="10">
-        <f t="shared" ref="K12:K19" si="6">J12*$D12</f>
-        <v>2.8571428571428568</v>
-      </c>
-      <c r="L12" s="5">
-        <v>4</v>
-      </c>
       <c r="M12" s="24">
-        <f t="shared" si="2"/>
-        <v>0.19047619047619047</v>
+        <f t="shared" ref="M12:M14" si="4">IF($E12="Y", L12/SUM($F12,$I12,$L12), (1/L12)/SUM(1/$F12,1/$I12,1/$L12))</f>
+        <v>0.24</v>
       </c>
       <c r="N12" s="10">
-        <f t="shared" ref="N12:N19" si="7">M12*$D12</f>
-        <v>2.8571428571428568</v>
-      </c>
-      <c r="O12" s="5">
-        <v>4</v>
-      </c>
-      <c r="P12" s="24">
-        <f t="shared" si="3"/>
-        <v>0.19047619047619047</v>
-      </c>
-      <c r="Q12" s="10">
-        <f t="shared" ref="Q12:Q19" si="8">P12*$D12</f>
-        <v>2.8571428571428568</v>
-      </c>
-      <c r="R12" s="5">
-        <v>4</v>
-      </c>
-      <c r="S12" s="24">
-        <f t="shared" si="4"/>
-        <v>0.19047619047619047</v>
-      </c>
-      <c r="T12" s="10">
-        <f t="shared" ref="T12:T19" si="9">S12*$D12</f>
-        <v>2.8571428571428568</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B13" s="55" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="56"/>
-      <c r="D13" s="23">
-        <v>10</v>
+        <f t="shared" ref="N12:N14" si="5">M12*D12</f>
+        <v>7.1999999999999993</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B13" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="57" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" s="24">
+        <v>30</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>15</v>
@@ -1585,522 +1490,121 @@
         <v>4</v>
       </c>
       <c r="G13" s="24">
-        <f t="shared" ref="G13:G19" si="10">IF($E13="Y", F13/SUM($F13,$I13,$L13,$O13,$R13), (1/F13)/SUM(1/$F13,1/$I13,1/$L13,1/$O13,1/$R13))</f>
-        <v>0.23529411764705882</v>
+        <f t="shared" si="0"/>
+        <v>0.22222222222222221</v>
       </c>
       <c r="H13" s="10">
+        <f t="shared" si="1"/>
+        <v>6.6666666666666661</v>
+      </c>
+      <c r="I13" s="5">
+        <v>8</v>
+      </c>
+      <c r="J13" s="24">
+        <f t="shared" si="2"/>
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="K13" s="10">
+        <f t="shared" si="3"/>
+        <v>13.333333333333332</v>
+      </c>
+      <c r="L13" s="5">
+        <v>6</v>
+      </c>
+      <c r="M13" s="24">
+        <f t="shared" si="4"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="N13" s="10">
         <f t="shared" si="5"/>
-        <v>2.3529411764705883</v>
-      </c>
-      <c r="I13" s="5">
-        <v>3</v>
-      </c>
-      <c r="J13" s="24">
-        <f t="shared" ref="J13:J19" si="11">IF($E13="Y", I13/SUM($F13,$I13,$L13,$O13,$R13), (1/I13)/SUM(1/$F13,1/$I13,1/$L13,1/$O13,1/$R13))</f>
-        <v>0.17647058823529413</v>
-      </c>
-      <c r="K13" s="10">
-        <f t="shared" si="6"/>
-        <v>1.7647058823529413</v>
-      </c>
-      <c r="L13" s="5">
-        <v>3</v>
-      </c>
-      <c r="M13" s="24">
-        <f t="shared" ref="M13:M19" si="12">IF($E13="Y", L13/SUM($F13,$I13,$L13,$O13,$R13), (1/L13)/SUM(1/$F13,1/$I13,1/$L13,1/$O13,1/$R13))</f>
-        <v>0.17647058823529413</v>
-      </c>
-      <c r="N13" s="10">
-        <f t="shared" si="7"/>
-        <v>1.7647058823529413</v>
-      </c>
-      <c r="O13" s="5">
-        <v>4</v>
-      </c>
-      <c r="P13" s="24">
-        <f t="shared" ref="P13:P19" si="13">IF($E13="Y", O13/SUM($F13,$I13,$L13,$O13,$R13), (1/O13)/SUM(1/$F13,1/$I13,1/$L13,1/$O13,1/$R13))</f>
-        <v>0.23529411764705882</v>
-      </c>
-      <c r="Q13" s="10">
-        <f t="shared" si="8"/>
-        <v>2.3529411764705883</v>
-      </c>
-      <c r="R13" s="5">
-        <v>3</v>
-      </c>
-      <c r="S13" s="24">
-        <f t="shared" ref="S13:S19" si="14">IF($E13="Y", R13/SUM($F13,$I13,$L13,$O13,$R13), (1/R13)/SUM(1/$F13,1/$I13,1/$L13,1/$O13,1/$R13))</f>
-        <v>0.17647058823529413</v>
-      </c>
-      <c r="T13" s="10">
-        <f t="shared" si="9"/>
-        <v>1.7647058823529413</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B14" s="55" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="56"/>
-      <c r="D14" s="23">
         <v>10</v>
       </c>
+    </row>
+    <row r="14" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="24">
+        <v>15</v>
+      </c>
       <c r="E14" s="10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F14" s="5">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="G14" s="24">
-        <f t="shared" si="10"/>
-        <v>0.22727272727272727</v>
+        <f t="shared" si="0"/>
+        <v>0.26829268292682923</v>
       </c>
       <c r="H14" s="10">
+        <f t="shared" si="1"/>
+        <v>4.0243902439024382</v>
+      </c>
+      <c r="I14" s="5">
+        <v>40</v>
+      </c>
+      <c r="J14" s="24">
+        <f t="shared" si="2"/>
+        <v>0.53658536585365846</v>
+      </c>
+      <c r="K14" s="10">
+        <f t="shared" si="3"/>
+        <v>8.0487804878048763</v>
+      </c>
+      <c r="L14" s="5">
+        <v>110</v>
+      </c>
+      <c r="M14" s="24">
+        <f t="shared" si="4"/>
+        <v>0.19512195121951215</v>
+      </c>
+      <c r="N14" s="10">
         <f t="shared" si="5"/>
-        <v>2.2727272727272725</v>
-      </c>
-      <c r="I14" s="5">
-        <v>5</v>
-      </c>
-      <c r="J14" s="24">
-        <f t="shared" si="11"/>
-        <v>0.22727272727272727</v>
-      </c>
-      <c r="K14" s="10">
-        <f t="shared" si="6"/>
-        <v>2.2727272727272725</v>
-      </c>
-      <c r="L14" s="5">
-        <v>4</v>
-      </c>
-      <c r="M14" s="24">
-        <f t="shared" si="12"/>
-        <v>0.18181818181818182</v>
-      </c>
-      <c r="N14" s="10">
-        <f t="shared" si="7"/>
-        <v>1.8181818181818183</v>
-      </c>
-      <c r="O14" s="5">
-        <v>4</v>
-      </c>
-      <c r="P14" s="24">
-        <f t="shared" si="13"/>
-        <v>0.18181818181818182</v>
-      </c>
-      <c r="Q14" s="10">
-        <f t="shared" si="8"/>
-        <v>1.8181818181818183</v>
-      </c>
-      <c r="R14" s="5">
-        <v>4</v>
-      </c>
-      <c r="S14" s="24">
-        <f t="shared" si="14"/>
-        <v>0.18181818181818182</v>
-      </c>
-      <c r="T14" s="10">
-        <f t="shared" si="9"/>
-        <v>1.8181818181818183</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B15" s="55" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="56"/>
-      <c r="D15" s="23">
-        <v>15</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F15" s="5">
-        <v>4</v>
-      </c>
-      <c r="G15" s="24">
-        <f t="shared" si="10"/>
-        <v>0.21052631578947367</v>
-      </c>
-      <c r="H15" s="10">
-        <f t="shared" si="5"/>
-        <v>3.1578947368421053</v>
-      </c>
-      <c r="I15" s="5">
-        <v>4</v>
-      </c>
-      <c r="J15" s="24">
-        <f t="shared" si="11"/>
-        <v>0.21052631578947367</v>
-      </c>
-      <c r="K15" s="10">
-        <f t="shared" si="6"/>
-        <v>3.1578947368421053</v>
-      </c>
-      <c r="L15" s="5">
-        <v>5</v>
-      </c>
-      <c r="M15" s="24">
-        <f t="shared" si="12"/>
-        <v>0.26315789473684209</v>
-      </c>
-      <c r="N15" s="10">
-        <f t="shared" si="7"/>
-        <v>3.9473684210526314</v>
-      </c>
-      <c r="O15" s="5">
-        <v>3</v>
-      </c>
-      <c r="P15" s="24">
-        <f t="shared" si="13"/>
-        <v>0.15789473684210525</v>
-      </c>
-      <c r="Q15" s="10">
-        <f t="shared" si="8"/>
-        <v>2.3684210526315788</v>
-      </c>
-      <c r="R15" s="5">
-        <v>3</v>
-      </c>
-      <c r="S15" s="24">
-        <f t="shared" si="14"/>
-        <v>0.15789473684210525</v>
-      </c>
-      <c r="T15" s="10">
-        <f t="shared" si="9"/>
-        <v>2.3684210526315788</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B16" s="55" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" s="56"/>
-      <c r="D16" s="23">
-        <v>10</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="5">
-        <v>3</v>
-      </c>
-      <c r="G16" s="24">
-        <f t="shared" si="10"/>
-        <v>0.17647058823529413</v>
-      </c>
-      <c r="H16" s="10">
-        <f t="shared" si="5"/>
-        <v>1.7647058823529413</v>
-      </c>
-      <c r="I16" s="5">
-        <v>5</v>
-      </c>
-      <c r="J16" s="24">
-        <f t="shared" si="11"/>
-        <v>0.29411764705882354</v>
-      </c>
-      <c r="K16" s="10">
-        <f t="shared" si="6"/>
-        <v>2.9411764705882355</v>
-      </c>
-      <c r="L16" s="5">
-        <v>3</v>
-      </c>
-      <c r="M16" s="24">
-        <f t="shared" si="12"/>
-        <v>0.17647058823529413</v>
-      </c>
-      <c r="N16" s="10">
-        <f t="shared" si="7"/>
-        <v>1.7647058823529413</v>
-      </c>
-      <c r="O16" s="5">
-        <v>3</v>
-      </c>
-      <c r="P16" s="24">
-        <f t="shared" si="13"/>
-        <v>0.17647058823529413</v>
-      </c>
-      <c r="Q16" s="10">
-        <f t="shared" si="8"/>
-        <v>1.7647058823529413</v>
-      </c>
-      <c r="R16" s="5">
-        <v>3</v>
-      </c>
-      <c r="S16" s="24">
-        <f t="shared" si="14"/>
-        <v>0.17647058823529413</v>
-      </c>
-      <c r="T16" s="10">
-        <f t="shared" si="9"/>
-        <v>1.7647058823529413</v>
-      </c>
-    </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B17" s="55" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="56"/>
-      <c r="D17" s="23">
-        <v>10</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" s="5">
-        <v>4</v>
-      </c>
-      <c r="G17" s="24">
-        <f t="shared" si="10"/>
-        <v>0.19047619047619047</v>
-      </c>
-      <c r="H17" s="10">
-        <f t="shared" si="5"/>
-        <v>1.9047619047619047</v>
-      </c>
-      <c r="I17" s="5">
-        <v>4</v>
-      </c>
-      <c r="J17" s="24">
-        <f t="shared" si="11"/>
-        <v>0.19047619047619047</v>
-      </c>
-      <c r="K17" s="10">
-        <f t="shared" si="6"/>
-        <v>1.9047619047619047</v>
-      </c>
-      <c r="L17" s="5">
-        <v>3</v>
-      </c>
-      <c r="M17" s="24">
-        <f t="shared" si="12"/>
-        <v>0.14285714285714285</v>
-      </c>
-      <c r="N17" s="10">
-        <f t="shared" si="7"/>
-        <v>1.4285714285714284</v>
-      </c>
-      <c r="O17" s="5">
-        <v>5</v>
-      </c>
-      <c r="P17" s="24">
-        <f t="shared" si="13"/>
-        <v>0.23809523809523808</v>
-      </c>
-      <c r="Q17" s="10">
-        <f t="shared" si="8"/>
-        <v>2.3809523809523809</v>
-      </c>
-      <c r="R17" s="5">
-        <v>5</v>
-      </c>
-      <c r="S17" s="24">
-        <f t="shared" si="14"/>
-        <v>0.23809523809523808</v>
-      </c>
-      <c r="T17" s="10">
-        <f t="shared" si="9"/>
-        <v>2.3809523809523809</v>
-      </c>
-    </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B18" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" s="56"/>
-      <c r="D18" s="23">
-        <v>5</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F18" s="5">
-        <v>3</v>
-      </c>
-      <c r="G18" s="24">
-        <f t="shared" si="10"/>
-        <v>0.17647058823529413</v>
-      </c>
-      <c r="H18" s="10">
-        <f t="shared" si="5"/>
-        <v>0.88235294117647067</v>
-      </c>
-      <c r="I18" s="5">
-        <v>4</v>
-      </c>
-      <c r="J18" s="24">
-        <f t="shared" si="11"/>
-        <v>0.23529411764705882</v>
-      </c>
-      <c r="K18" s="10">
-        <f t="shared" si="6"/>
-        <v>1.1764705882352942</v>
-      </c>
-      <c r="L18" s="5">
-        <v>1</v>
-      </c>
-      <c r="M18" s="24">
-        <f t="shared" si="12"/>
-        <v>5.8823529411764705E-2</v>
-      </c>
-      <c r="N18" s="10">
-        <f t="shared" si="7"/>
-        <v>0.29411764705882354</v>
-      </c>
-      <c r="O18" s="5">
-        <v>4</v>
-      </c>
-      <c r="P18" s="24">
-        <f t="shared" si="13"/>
-        <v>0.23529411764705882</v>
-      </c>
-      <c r="Q18" s="10">
-        <f t="shared" si="8"/>
-        <v>1.1764705882352942</v>
-      </c>
-      <c r="R18" s="5">
-        <v>5</v>
-      </c>
-      <c r="S18" s="24">
-        <f t="shared" si="14"/>
-        <v>0.29411764705882354</v>
-      </c>
-      <c r="T18" s="10">
-        <f t="shared" si="9"/>
-        <v>1.4705882352941178</v>
-      </c>
-    </row>
-    <row r="19" spans="2:20" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="29"/>
-      <c r="D19" s="23">
-        <v>5</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F19" s="6">
-        <v>4</v>
-      </c>
-      <c r="G19" s="25">
-        <f t="shared" si="10"/>
-        <v>0.22222222222222221</v>
-      </c>
-      <c r="H19" s="10">
-        <f t="shared" si="5"/>
-        <v>1.1111111111111112</v>
-      </c>
-      <c r="I19" s="6">
-        <v>4</v>
-      </c>
-      <c r="J19" s="25">
-        <f t="shared" si="11"/>
-        <v>0.22222222222222221</v>
-      </c>
-      <c r="K19" s="10">
-        <f t="shared" si="6"/>
-        <v>1.1111111111111112</v>
-      </c>
-      <c r="L19" s="6">
-        <v>4</v>
-      </c>
-      <c r="M19" s="25">
-        <f t="shared" si="12"/>
-        <v>0.22222222222222221</v>
-      </c>
-      <c r="N19" s="10">
-        <f t="shared" si="7"/>
-        <v>1.1111111111111112</v>
-      </c>
-      <c r="O19" s="6">
-        <v>3</v>
-      </c>
-      <c r="P19" s="25">
-        <f t="shared" si="13"/>
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="Q19" s="10">
-        <f t="shared" si="8"/>
-        <v>0.83333333333333326</v>
-      </c>
-      <c r="R19" s="6">
-        <v>3</v>
-      </c>
-      <c r="S19" s="25">
-        <f t="shared" si="14"/>
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="T19" s="10">
-        <f t="shared" si="9"/>
-        <v>0.83333333333333326</v>
-      </c>
-    </row>
-    <row r="20" spans="2:20" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="41" t="s">
+        <v>2.926829268292682</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="43"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="27">
-        <f>SUM(H11:H19)</f>
-        <v>21.228449912660441</v>
-      </c>
-      <c r="I20" s="13"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="27">
-        <f>SUM(K11:K19)</f>
-        <v>20.343885560603827</v>
-      </c>
-      <c r="L20" s="13"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="27">
-        <f>SUM(N11:N19)</f>
-        <v>18.143799784666658</v>
-      </c>
-      <c r="O20" s="13"/>
-      <c r="P20" s="14"/>
-      <c r="Q20" s="27">
-        <f>SUM(Q11:Q19)</f>
-        <v>20.81530698403763</v>
-      </c>
-      <c r="R20" s="13"/>
-      <c r="S20" s="14"/>
-      <c r="T20" s="27">
-        <f>SUM(T11:T19)</f>
-        <v>19.468557758031441</v>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="27">
+        <f>SUM(H11:H14)</f>
+        <v>24.35772357723577</v>
+      </c>
+      <c r="I15" s="13"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="27">
+        <f>SUM(K11:K14)</f>
+        <v>38.848780487804873</v>
+      </c>
+      <c r="L15" s="13"/>
+      <c r="M15" s="14"/>
+      <c r="N15" s="27">
+        <f>SUM(N11:N14)</f>
+        <v>36.793495934959338</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="B20:E20"/>
+  <mergeCells count="10">
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
     <mergeCell ref="I9:K9"/>
     <mergeCell ref="L9:N9"/>
-    <mergeCell ref="O9:Q9"/>
-    <mergeCell ref="R9:T9"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="F9:H9"/>
+    <mergeCell ref="B15:E15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2197,22 +1701,22 @@
     </row>
     <row r="15" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="57" t="s">
+      <c r="B16" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="58"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="59"/>
-      <c r="F16" s="60" t="s">
+      <c r="C16" s="54"/>
+      <c r="D16" s="54"/>
+      <c r="E16" s="55"/>
+      <c r="F16" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="61"/>
-      <c r="H16" s="62"/>
-      <c r="I16" s="30" t="s">
+      <c r="G16" s="41"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="J16" s="31"/>
-      <c r="K16" s="32"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="34"/>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B17" s="8" t="s">
@@ -2319,12 +1823,12 @@
       </c>
     </row>
     <row r="20" spans="2:11" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="41" t="s">
+      <c r="B20" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="43"/>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="45"/>
       <c r="F20" s="13"/>
       <c r="G20" s="14"/>
       <c r="H20" s="27">
@@ -2355,6 +1859,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="37bd234a-b872-4d8f-a05f-9ce9a06b0a24" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="619bfd31-fbc9-4e3d-b639-5680fd0427c3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100445E206EC97B5241AE364FC742D190F1" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8284591227d7a4ff90c48262bf6356f1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="619bfd31-fbc9-4e3d-b639-5680fd0427c3" xmlns:ns3="37bd234a-b872-4d8f-a05f-9ce9a06b0a24" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b29a3fb53242aaf6387bf4e700398a19" ns2:_="" ns3:_="">
     <xsd:import namespace="619bfd31-fbc9-4e3d-b639-5680fd0427c3"/>
@@ -2609,27 +2133,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="37bd234a-b872-4d8f-a05f-9ce9a06b0a24" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="619bfd31-fbc9-4e3d-b639-5680fd0427c3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3A021D7-EA7F-46DD-AD48-5861691E078E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="619bfd31-fbc9-4e3d-b639-5680fd0427c3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="37bd234a-b872-4d8f-a05f-9ce9a06b0a24"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1748E98C-71FF-4E5A-BAD7-3F9220D62AE3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F6E05F-13AA-425A-905B-6BF8E82F9AC9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2646,29 +2175,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3A021D7-EA7F-46DD-AD48-5861691E078E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="619bfd31-fbc9-4e3d-b639-5680fd0427c3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="37bd234a-b872-4d8f-a05f-9ce9a06b0a24"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1748E98C-71FF-4E5A-BAD7-3F9220D62AE3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>